<commit_message>
finished wiring inner units, sequencer
</commit_message>
<xml_diff>
--- a/unit interface.xlsx
+++ b/unit interface.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9656EF4F-6361-4945-B172-A838FF58BE53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3EF98E-9275-4390-ABC8-52AE0562991B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -434,24 +434,9 @@
     <t>low for write mode</t>
   </si>
   <si>
-    <t>NOT_OPDC_11111</t>
-  </si>
-  <si>
-    <t>NOT_OPDC_10101</t>
-  </si>
-  <si>
     <t xml:space="preserve">IO unit (here: 0) </t>
   </si>
   <si>
-    <t>NOT_OPDC_11000</t>
-  </si>
-  <si>
-    <t>NOT_OPDC_11001</t>
-  </si>
-  <si>
-    <t>NOT_OPDC_11010</t>
-  </si>
-  <si>
     <t>DATA0-DATA7</t>
   </si>
   <si>
@@ -465,6 +450,21 @@
   </si>
   <si>
     <t>induces write on rising, pop on falling if corresponding operation is active</t>
+  </si>
+  <si>
+    <t>NOT_OPCD_10101</t>
+  </si>
+  <si>
+    <t>NOT_OPCD_11111</t>
+  </si>
+  <si>
+    <t>NOT_OPCD_11000</t>
+  </si>
+  <si>
+    <t>NOT_OPCD_11001</t>
+  </si>
+  <si>
+    <t>NOT_OPCD_11010</t>
   </si>
 </sst>
 </file>
@@ -671,7 +671,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -703,24 +703,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -731,29 +745,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -763,12 +756,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1095,10 +1082,10 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="20" t="s">
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
@@ -1118,9 +1105,9 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A3" s="33"/>
-      <c r="B3" s="32"/>
-      <c r="C3" s="33" t="s">
+      <c r="A3" s="23"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="23" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -1135,9 +1122,9 @@
       <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A4" s="33"/>
-      <c r="B4" s="32"/>
-      <c r="C4" s="33"/>
+      <c r="A4" s="23"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="23"/>
       <c r="D4" s="2" t="s">
         <v>9</v>
       </c>
@@ -1150,9 +1137,9 @@
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A5" s="33"/>
-      <c r="B5" s="32"/>
-      <c r="C5" s="33"/>
+      <c r="A5" s="23"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="23"/>
       <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
@@ -1165,9 +1152,9 @@
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A6" s="33"/>
-      <c r="B6" s="32"/>
-      <c r="C6" s="33"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="23"/>
       <c r="D6" s="2" t="s">
         <v>11</v>
       </c>
@@ -1180,8 +1167,8 @@
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A7" s="33"/>
-      <c r="B7" s="32" t="s">
+      <c r="A7" s="23"/>
+      <c r="B7" s="21" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -1199,9 +1186,9 @@
       <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A8" s="33"/>
-      <c r="B8" s="32"/>
-      <c r="C8" s="33" t="s">
+      <c r="A8" s="23"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="23" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="2" t="s">
@@ -1216,9 +1203,9 @@
       <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A9" s="33"/>
-      <c r="B9" s="32"/>
-      <c r="C9" s="33"/>
+      <c r="A9" s="23"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="23"/>
       <c r="D9" s="2" t="s">
         <v>22</v>
       </c>
@@ -1231,9 +1218,9 @@
       <c r="G9" s="2"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A10" s="33"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="33"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="23"/>
       <c r="D10" s="2" t="s">
         <v>23</v>
       </c>
@@ -1246,9 +1233,9 @@
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A11" s="33"/>
-      <c r="B11" s="32"/>
-      <c r="C11" s="33"/>
+      <c r="A11" s="23"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="23"/>
       <c r="D11" s="2" t="s">
         <v>24</v>
       </c>
@@ -1261,8 +1248,8 @@
       <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A12" s="33"/>
-      <c r="B12" s="32" t="s">
+      <c r="A12" s="23"/>
+      <c r="B12" s="21" t="s">
         <v>25</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -1280,9 +1267,9 @@
       <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A13" s="33"/>
-      <c r="B13" s="32"/>
-      <c r="C13" s="33" t="s">
+      <c r="A13" s="23"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="23" t="s">
         <v>13</v>
       </c>
       <c r="D13" s="2" t="s">
@@ -1297,9 +1284,9 @@
       <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A14" s="33"/>
-      <c r="B14" s="32"/>
-      <c r="C14" s="33"/>
+      <c r="A14" s="23"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="23"/>
       <c r="D14" s="2" t="s">
         <v>28</v>
       </c>
@@ -1312,9 +1299,9 @@
       <c r="G14" s="2"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A15" s="33"/>
-      <c r="B15" s="32"/>
-      <c r="C15" s="33"/>
+      <c r="A15" s="23"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="23"/>
       <c r="D15" s="2" t="s">
         <v>29</v>
       </c>
@@ -1327,9 +1314,9 @@
       <c r="G15" s="2"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A16" s="33"/>
-      <c r="B16" s="32"/>
-      <c r="C16" s="33"/>
+      <c r="A16" s="23"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="23"/>
       <c r="D16" s="2" t="s">
         <v>30</v>
       </c>
@@ -1342,8 +1329,8 @@
       <c r="G16" s="2"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A17" s="33"/>
-      <c r="B17" s="32" t="s">
+      <c r="A17" s="23"/>
+      <c r="B17" s="21" t="s">
         <v>31</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -1361,9 +1348,9 @@
       <c r="G17" s="2"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A18" s="33"/>
-      <c r="B18" s="32"/>
-      <c r="C18" s="33" t="s">
+      <c r="A18" s="23"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="23" t="s">
         <v>13</v>
       </c>
       <c r="D18" s="2" t="s">
@@ -1378,9 +1365,9 @@
       <c r="G18" s="2"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A19" s="33"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="33"/>
+      <c r="A19" s="23"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="23"/>
       <c r="D19" s="2" t="s">
         <v>34</v>
       </c>
@@ -1393,9 +1380,9 @@
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A20" s="33"/>
-      <c r="B20" s="32"/>
-      <c r="C20" s="33"/>
+      <c r="A20" s="23"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="23"/>
       <c r="D20" s="2" t="s">
         <v>35</v>
       </c>
@@ -1408,9 +1395,9 @@
       <c r="G20" s="2"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A21" s="33"/>
-      <c r="B21" s="32"/>
-      <c r="C21" s="33"/>
+      <c r="A21" s="23"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="23"/>
       <c r="D21" s="2" t="s">
         <v>36</v>
       </c>
@@ -1423,11 +1410,11 @@
       <c r="G21" s="2"/>
     </row>
     <row r="22" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="33"/>
-      <c r="B22" s="37" t="s">
+      <c r="A22" s="23"/>
+      <c r="B22" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="C22" s="30" t="s">
         <v>56</v>
       </c>
       <c r="D22" s="2" t="s">
@@ -1442,9 +1429,9 @@
       <c r="G22" s="2"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A23" s="33"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="28"/>
+      <c r="A23" s="23"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="32"/>
       <c r="D23" s="2" t="s">
         <v>48</v>
       </c>
@@ -1457,9 +1444,9 @@
       <c r="G23" s="2"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A24" s="33"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="26" t="s">
+      <c r="A24" s="23"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="30" t="s">
         <v>57</v>
       </c>
       <c r="D24" s="2" t="s">
@@ -1474,9 +1461,9 @@
       <c r="G24" s="2"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A25" s="33"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="28"/>
+      <c r="A25" s="23"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="32"/>
       <c r="D25" s="2" t="s">
         <v>49</v>
       </c>
@@ -1489,9 +1476,9 @@
       <c r="G25" s="2"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A26" s="33"/>
-      <c r="B26" s="38"/>
-      <c r="C26" s="26" t="s">
+      <c r="A26" s="23"/>
+      <c r="B26" s="35"/>
+      <c r="C26" s="30" t="s">
         <v>58</v>
       </c>
       <c r="D26" s="2" t="s">
@@ -1506,9 +1493,9 @@
       <c r="G26" s="2"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A27" s="33"/>
-      <c r="B27" s="38"/>
-      <c r="C27" s="28"/>
+      <c r="A27" s="23"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="32"/>
       <c r="D27" s="2" t="s">
         <v>54</v>
       </c>
@@ -1521,8 +1508,8 @@
       <c r="G27" s="2"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A28" s="33"/>
-      <c r="B28" s="38"/>
+      <c r="A28" s="23"/>
+      <c r="B28" s="35"/>
       <c r="C28" s="4" t="s">
         <v>74</v>
       </c>
@@ -1540,8 +1527,8 @@
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A29" s="33"/>
-      <c r="B29" s="39"/>
+      <c r="A29" s="23"/>
+      <c r="B29" s="36"/>
       <c r="C29" s="4" t="s">
         <v>75</v>
       </c>
@@ -1559,7 +1546,7 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A30" s="33"/>
+      <c r="A30" s="23"/>
       <c r="B30" s="2" t="s">
         <v>37</v>
       </c>
@@ -1576,7 +1563,7 @@
       <c r="G30" s="2"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A31" s="33"/>
+      <c r="A31" s="23"/>
       <c r="B31" s="2" t="s">
         <v>38</v>
       </c>
@@ -1593,7 +1580,7 @@
       <c r="G31" s="2"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A32" s="33"/>
+      <c r="A32" s="23"/>
       <c r="B32" s="2" t="s">
         <v>39</v>
       </c>
@@ -1610,7 +1597,7 @@
       <c r="G32" s="2"/>
     </row>
     <row r="33" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A33" s="35"/>
+      <c r="A33" s="26"/>
       <c r="B33" s="3" t="s">
         <v>40</v>
       </c>
@@ -1627,10 +1614,10 @@
       <c r="G33" s="3"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A34" s="24" t="s">
+      <c r="A34" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="B34" s="31" t="s">
+      <c r="B34" s="28" t="s">
         <v>65</v>
       </c>
       <c r="C34" s="5" t="s">
@@ -1650,9 +1637,9 @@
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A35" s="24"/>
-      <c r="B35" s="41"/>
-      <c r="C35" s="33" t="s">
+      <c r="A35" s="25"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="23" t="s">
         <v>67</v>
       </c>
       <c r="D35" s="2" t="s">
@@ -1669,9 +1656,9 @@
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A36" s="24"/>
-      <c r="B36" s="41"/>
-      <c r="C36" s="33"/>
+      <c r="A36" s="25"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="23"/>
       <c r="D36" s="2" t="s">
         <v>61</v>
       </c>
@@ -1684,9 +1671,9 @@
       <c r="G36" s="2"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A37" s="24"/>
-      <c r="B37" s="41"/>
-      <c r="C37" s="33" t="s">
+      <c r="A37" s="25"/>
+      <c r="B37" s="29"/>
+      <c r="C37" s="23" t="s">
         <v>66</v>
       </c>
       <c r="D37" s="2" t="s">
@@ -1701,9 +1688,9 @@
       <c r="G37" s="2"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A38" s="24"/>
-      <c r="B38" s="41"/>
-      <c r="C38" s="33"/>
+      <c r="A38" s="25"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="23"/>
       <c r="D38" s="2" t="s">
         <v>63</v>
       </c>
@@ -1716,11 +1703,11 @@
       <c r="G38" s="2"/>
     </row>
     <row r="39" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A39" s="24"/>
-      <c r="B39" s="32" t="s">
+      <c r="A39" s="25"/>
+      <c r="B39" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="C39" s="32" t="s">
+      <c r="C39" s="21" t="s">
         <v>56</v>
       </c>
       <c r="D39" s="2" t="s">
@@ -1735,9 +1722,9 @@
       <c r="G39" s="2"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A40" s="24"/>
-      <c r="B40" s="32"/>
-      <c r="C40" s="32"/>
+      <c r="A40" s="25"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
       <c r="D40" s="2" t="s">
         <v>48</v>
       </c>
@@ -1750,9 +1737,9 @@
       <c r="G40" s="2"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A41" s="24"/>
-      <c r="B41" s="32"/>
-      <c r="C41" s="32" t="s">
+      <c r="A41" s="25"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="21" t="s">
         <v>57</v>
       </c>
       <c r="D41" s="2" t="s">
@@ -1767,9 +1754,9 @@
       <c r="G41" s="2"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A42" s="24"/>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
+      <c r="A42" s="25"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
       <c r="D42" s="2" t="s">
         <v>49</v>
       </c>
@@ -1782,8 +1769,8 @@
       <c r="G42" s="2"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A43" s="24"/>
-      <c r="B43" s="33" t="s">
+      <c r="A43" s="25"/>
+      <c r="B43" s="23" t="s">
         <v>37</v>
       </c>
       <c r="C43" s="2" t="s">
@@ -1801,8 +1788,8 @@
       <c r="G43" s="2"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A44" s="24"/>
-      <c r="B44" s="33"/>
+      <c r="A44" s="25"/>
+      <c r="B44" s="23"/>
       <c r="C44" s="2" t="s">
         <v>68</v>
       </c>
@@ -1818,7 +1805,7 @@
       <c r="G44" s="2"/>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A45" s="24"/>
+      <c r="A45" s="25"/>
       <c r="B45" s="2" t="s">
         <v>38</v>
       </c>
@@ -1835,7 +1822,7 @@
       <c r="G45" s="2"/>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A46" s="24"/>
+      <c r="A46" s="25"/>
       <c r="B46" s="2" t="s">
         <v>39</v>
       </c>
@@ -1852,7 +1839,7 @@
       <c r="G46" s="2"/>
     </row>
     <row r="47" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A47" s="25"/>
+      <c r="A47" s="27"/>
       <c r="B47" s="3" t="s">
         <v>70</v>
       </c>
@@ -1869,10 +1856,10 @@
       <c r="G47" s="3"/>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A48" s="40" t="s">
+      <c r="A48" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B48" s="36" t="s">
+      <c r="B48" s="20" t="s">
         <v>97</v>
       </c>
       <c r="C48" s="7" t="s">
@@ -1895,9 +1882,9 @@
       <c r="J48" s="15"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A49" s="24"/>
-      <c r="B49" s="32"/>
-      <c r="C49" s="33" t="s">
+      <c r="A49" s="25"/>
+      <c r="B49" s="21"/>
+      <c r="C49" s="23" t="s">
         <v>87</v>
       </c>
       <c r="D49" s="2" t="s">
@@ -1915,9 +1902,9 @@
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A50" s="24"/>
-      <c r="B50" s="32"/>
-      <c r="C50" s="33"/>
+      <c r="A50" s="25"/>
+      <c r="B50" s="21"/>
+      <c r="C50" s="23"/>
       <c r="D50" s="2" t="s">
         <v>85</v>
       </c>
@@ -1933,8 +1920,8 @@
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A51" s="24"/>
-      <c r="B51" s="32"/>
+      <c r="A51" s="25"/>
+      <c r="B51" s="21"/>
       <c r="C51" s="2" t="s">
         <v>91</v>
       </c>
@@ -1953,9 +1940,9 @@
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A52" s="24"/>
-      <c r="B52" s="32"/>
-      <c r="C52" s="33" t="s">
+      <c r="A52" s="25"/>
+      <c r="B52" s="21"/>
+      <c r="C52" s="23" t="s">
         <v>92</v>
       </c>
       <c r="D52" s="2" t="s">
@@ -1975,9 +1962,9 @@
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A53" s="24"/>
-      <c r="B53" s="32"/>
-      <c r="C53" s="33"/>
+      <c r="A53" s="25"/>
+      <c r="B53" s="21"/>
+      <c r="C53" s="23"/>
       <c r="D53" s="2" t="s">
         <v>89</v>
       </c>
@@ -1995,9 +1982,9 @@
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A54" s="24"/>
-      <c r="B54" s="32"/>
-      <c r="C54" s="33" t="s">
+      <c r="A54" s="25"/>
+      <c r="B54" s="21"/>
+      <c r="C54" s="23" t="s">
         <v>94</v>
       </c>
       <c r="D54" s="2" t="s">
@@ -2015,9 +2002,9 @@
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A55" s="24"/>
-      <c r="B55" s="32"/>
-      <c r="C55" s="33"/>
+      <c r="A55" s="25"/>
+      <c r="B55" s="21"/>
+      <c r="C55" s="23"/>
       <c r="D55" s="2" t="s">
         <v>95</v>
       </c>
@@ -2037,8 +2024,8 @@
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A56" s="24"/>
-      <c r="B56" s="33" t="s">
+      <c r="A56" s="25"/>
+      <c r="B56" s="23" t="s">
         <v>102</v>
       </c>
       <c r="C56" s="2" t="s">
@@ -2059,9 +2046,9 @@
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A57" s="24"/>
-      <c r="B57" s="33"/>
-      <c r="C57" s="33" t="s">
+      <c r="A57" s="25"/>
+      <c r="B57" s="23"/>
+      <c r="C57" s="23" t="s">
         <v>100</v>
       </c>
       <c r="D57" s="2" t="s">
@@ -2079,9 +2066,9 @@
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A58" s="24"/>
-      <c r="B58" s="33"/>
-      <c r="C58" s="33"/>
+      <c r="A58" s="25"/>
+      <c r="B58" s="23"/>
+      <c r="C58" s="23"/>
       <c r="D58" s="2" t="s">
         <v>42</v>
       </c>
@@ -2099,9 +2086,9 @@
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A59" s="24"/>
-      <c r="B59" s="33"/>
-      <c r="C59" s="33"/>
+      <c r="A59" s="25"/>
+      <c r="B59" s="23"/>
+      <c r="C59" s="23"/>
       <c r="D59" s="2" t="s">
         <v>43</v>
       </c>
@@ -2119,8 +2106,8 @@
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A60" s="24"/>
-      <c r="B60" s="33"/>
+      <c r="A60" s="25"/>
+      <c r="B60" s="23"/>
       <c r="C60" s="8" t="s">
         <v>101</v>
       </c>
@@ -2139,13 +2126,13 @@
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A61" s="24"/>
-      <c r="B61" s="33"/>
+      <c r="A61" s="25"/>
+      <c r="B61" s="23"/>
       <c r="C61" s="8" t="s">
         <v>103</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>51</v>
@@ -2161,8 +2148,8 @@
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A62" s="24"/>
-      <c r="B62" s="33"/>
+      <c r="A62" s="25"/>
+      <c r="B62" s="23"/>
       <c r="C62" s="2" t="s">
         <v>14</v>
       </c>
@@ -2187,7 +2174,7 @@
       </c>
     </row>
     <row r="63" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A63" s="25"/>
+      <c r="A63" s="27"/>
       <c r="B63" s="12" t="s">
         <v>115</v>
       </c>
@@ -2214,7 +2201,7 @@
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A64" s="34" t="s">
+      <c r="A64" s="22" t="s">
         <v>111</v>
       </c>
       <c r="B64" s="11" t="s">
@@ -2238,7 +2225,7 @@
       </c>
     </row>
     <row r="65" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A65" s="35"/>
+      <c r="A65" s="26"/>
       <c r="B65" s="12" t="s">
         <v>115</v>
       </c>
@@ -2263,13 +2250,13 @@
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A66" s="40" t="s">
+      <c r="A66" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="B66" s="36" t="s">
+      <c r="B66" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="C66" s="34" t="s">
+      <c r="C66" s="22" t="s">
         <v>126</v>
       </c>
       <c r="D66" s="7" t="s">
@@ -2287,9 +2274,9 @@
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A67" s="24"/>
-      <c r="B67" s="32"/>
-      <c r="C67" s="33"/>
+      <c r="A67" s="25"/>
+      <c r="B67" s="21"/>
+      <c r="C67" s="23"/>
       <c r="D67" s="2" t="s">
         <v>119</v>
       </c>
@@ -2305,9 +2292,9 @@
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A68" s="24"/>
-      <c r="B68" s="32"/>
-      <c r="C68" s="33"/>
+      <c r="A68" s="25"/>
+      <c r="B68" s="21"/>
+      <c r="C68" s="23"/>
       <c r="D68" s="2" t="s">
         <v>110</v>
       </c>
@@ -2323,9 +2310,9 @@
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A69" s="24"/>
-      <c r="B69" s="32"/>
-      <c r="C69" s="33"/>
+      <c r="A69" s="25"/>
+      <c r="B69" s="21"/>
+      <c r="C69" s="23"/>
       <c r="D69" s="2" t="s">
         <v>120</v>
       </c>
@@ -2343,9 +2330,9 @@
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A70" s="24"/>
-      <c r="B70" s="32"/>
-      <c r="C70" s="33"/>
+      <c r="A70" s="25"/>
+      <c r="B70" s="21"/>
+      <c r="C70" s="23"/>
       <c r="D70" s="2" t="s">
         <v>121</v>
       </c>
@@ -2363,8 +2350,8 @@
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A71" s="24"/>
-      <c r="B71" s="32"/>
+      <c r="A71" s="25"/>
+      <c r="B71" s="21"/>
       <c r="C71" s="8" t="s">
         <v>127</v>
       </c>
@@ -2389,8 +2376,8 @@
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A72" s="24"/>
-      <c r="B72" s="32" t="s">
+      <c r="A72" s="25"/>
+      <c r="B72" s="21" t="s">
         <v>65</v>
       </c>
       <c r="C72" s="9" t="s">
@@ -2413,13 +2400,13 @@
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A73" s="24"/>
-      <c r="B73" s="32"/>
+      <c r="A73" s="25"/>
+      <c r="B73" s="21"/>
       <c r="C73" s="2" t="s">
         <v>128</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>51</v>
@@ -2434,22 +2421,22 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A74" s="24"/>
-      <c r="B74" s="19" t="s">
+    <row r="74" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A74" s="27"/>
+      <c r="B74" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="C74" s="20"/>
-      <c r="D74" s="21" t="s">
+      <c r="C74" s="10"/>
+      <c r="D74" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E74" s="21" t="s">
+      <c r="E74" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="F74" s="21" t="s">
+      <c r="F74" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="G74" s="21"/>
+      <c r="G74" s="3"/>
       <c r="H74" s="16">
         <v>2</v>
       </c>
@@ -2463,35 +2450,35 @@
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A75" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="B75" s="26" t="s">
+      <c r="A75" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="B75" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="C75" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="D75" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="C75" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F75" s="2" t="s">
+      <c r="E75" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F75" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="G75" s="2"/>
+      <c r="G75" s="5"/>
       <c r="H75" s="18">
         <v>1</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A76" s="24"/>
-      <c r="B76" s="27"/>
-      <c r="C76" s="30"/>
+      <c r="A76" s="25"/>
+      <c r="B76" s="31"/>
+      <c r="C76" s="33"/>
       <c r="D76" s="2" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>51</v>
@@ -2505,11 +2492,11 @@
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A77" s="24"/>
-      <c r="B77" s="27"/>
-      <c r="C77" s="30"/>
+      <c r="A77" s="25"/>
+      <c r="B77" s="31"/>
+      <c r="C77" s="33"/>
       <c r="D77" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>51</v>
@@ -2523,9 +2510,9 @@
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A78" s="24"/>
-      <c r="B78" s="27"/>
-      <c r="C78" s="31"/>
+      <c r="A78" s="25"/>
+      <c r="B78" s="31"/>
+      <c r="C78" s="28"/>
       <c r="D78" s="2" t="s">
         <v>110</v>
       </c>
@@ -2533,26 +2520,26 @@
         <v>51</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="H78" s="18">
         <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A79" s="24"/>
-      <c r="B79" s="28"/>
+      <c r="A79" s="25"/>
+      <c r="B79" s="32"/>
       <c r="C79" s="8" t="s">
         <v>45</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>45</v>
@@ -2567,11 +2554,11 @@
       </c>
     </row>
     <row r="80" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A80" s="25"/>
+      <c r="A80" s="27"/>
       <c r="B80" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="C80" s="22"/>
+      <c r="C80" s="19"/>
       <c r="D80" s="3" t="s">
         <v>114</v>
       </c>
@@ -2596,26 +2583,6 @@
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="B66:B71"/>
-    <mergeCell ref="B72:B73"/>
-    <mergeCell ref="C66:C70"/>
-    <mergeCell ref="A66:A74"/>
-    <mergeCell ref="A64:A65"/>
-    <mergeCell ref="A48:A63"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="A34:A47"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="C37:C38"/>
-    <mergeCell ref="B39:B42"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="B43:B44"/>
-    <mergeCell ref="C57:C59"/>
-    <mergeCell ref="B56:B62"/>
-    <mergeCell ref="C49:C50"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="B48:B55"/>
     <mergeCell ref="A75:A80"/>
     <mergeCell ref="B75:B79"/>
     <mergeCell ref="C75:C78"/>
@@ -2632,6 +2599,26 @@
     <mergeCell ref="C24:C25"/>
     <mergeCell ref="C26:C27"/>
     <mergeCell ref="B22:B29"/>
+    <mergeCell ref="A48:A63"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="A34:A47"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="C37:C38"/>
+    <mergeCell ref="B39:B42"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="B43:B44"/>
+    <mergeCell ref="C57:C59"/>
+    <mergeCell ref="B56:B62"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="B48:B55"/>
+    <mergeCell ref="B66:B71"/>
+    <mergeCell ref="B72:B73"/>
+    <mergeCell ref="C66:C70"/>
+    <mergeCell ref="A66:A74"/>
+    <mergeCell ref="A64:A65"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>